<commit_message>
docs: add JS snippet + insertion point per event, plus full implementation guide
Plan sheet now has two extra columns ready for the dev:
- Snippet JS: literal track(...) call to copy-paste
- Punto de inserción: semantic location (handler/effect/component)

Full implementation guide added at analytics/ANALYTICS.md, covering:
- Helper analytics.js (track, sha256, identify, toGA4Item, getGaClientId)
- Consent Mode v2 (denied default for ES, granted for MX)
- GTM bootstrap
- Country detection
- Per-component snippets for ANL-2 to ANL-8
- Server-side: GA4 Measurement Protocol + Meta CAPI with deduplication
- GTM/GA4 config: variables, triggers, tags, key events, custom dimensions, audiences
- QA: GTM Preview, GA4 DebugView, PR checklist

xlsx regenerated with new columns and adjusted widths.

https://claude.ai/code/session_01LtsMmom9oY6wGnqUbdTtQB
</commit_message>
<xml_diff>
--- a/analytics/equipzilla_events_plan.xlsx
+++ b/analytics/equipzilla_events_plan.xlsx
@@ -207,9 +207,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tbl_Plan" displayName="tbl_Plan" ref="A1:L29" headerRowCount="1">
-  <autoFilter ref="A1:L29"/>
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tbl_Plan" displayName="tbl_Plan" ref="A1:N29" headerRowCount="1">
+  <autoFilter ref="A1:N29"/>
+  <tableColumns count="14">
     <tableColumn id="1" name="Bloque"/>
     <tableColumn id="2" name="Evento (event_name)"/>
     <tableColumn id="3" name="Cuándo se dispara"/>
@@ -222,6 +222,8 @@
     <tableColumn id="10" name="Estado"/>
     <tableColumn id="11" name="Validado DebugView"/>
     <tableColumn id="12" name="Notas"/>
+    <tableColumn id="13" name="Snippet JS"/>
+    <tableColumn id="14" name="Punto de inserción"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -684,21 +686,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="60" customWidth="1" min="13" max="13"/>
+    <col width="56" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -762,6 +766,16 @@
           <t>Notas</t>
         </is>
       </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
+          <t>Snippet JS</t>
+        </is>
+      </c>
+      <c r="N1" s="3" t="inlineStr">
+        <is>
+          <t>Punto de inserción</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -824,6 +838,16 @@
           <t>Sustituye al "Búsqueda Realizada en la Home". Mandar también con results_count=0 para detectar consultas sin match.</t>
         </is>
       </c>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t>track('search', { search_term: query, results_count: results.length, search_location: 'home' });</t>
+        </is>
+      </c>
+      <c r="N2" s="4" t="inlineStr">
+        <is>
+          <t>Componente del buscador home: dentro del handler onSearch/onSubmit, tras recibir la respuesta de la API de búsqueda.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -886,6 +910,16 @@
           <t>Sustituye al "Resultado de Búsqueda Seleccionado".</t>
         </is>
       </c>
+      <c r="M3" s="4" t="inlineStr">
+        <is>
+          <t>track('select_search_result', { search_term: query, item_name: result.name, position: idx });</t>
+        </is>
+      </c>
+      <c r="N3" s="4" t="inlineStr">
+        <is>
+          <t>onClick de cada resultado/sugerencia, antes de la navegación.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -948,6 +982,16 @@
           <t>Sustituye al "Resultado de Búsqueda Eliminado".</t>
         </is>
       </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>track('search_clear', { search_term: previousQuery });</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>Handler onClear/onReset del buscador, antes de vaciar el state.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -1010,6 +1054,16 @@
           <t>Primer paso antes de elegir país.</t>
         </is>
       </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>track('whatsapp_widget_open');</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>onClick del botón flotante de WhatsApp, cuando pasa a estado open=true.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1072,6 +1126,16 @@
           <t>Unifica los dos eventos actuales (España y México) en uno con parámetro country.</t>
         </is>
       </c>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>track('whatsapp_country_click', { country: 'es' });</t>
+        </is>
+      </c>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t>onClick del enlace wa.me/&lt;numero&gt; de cada país, antes de la redirección.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1134,6 +1198,16 @@
           <t>Reemplaza al "Formulario OnlyPhone Visto". Aplica a todos los formularios para medir abandono. NO disparar un evento por cada cambio de campo.</t>
         </is>
       </c>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t>if (!startedRef.current) { track('form_start', { form_id: 'contact', form_location: 'home' }); startedRef.current = true; }</t>
+        </is>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>onFocus del primer input. Usar un useRef o flag local para que se dispare UNA vez por instancia del formulario.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1196,6 +1270,16 @@
           <t>Sustituye al "Error al Enviar Formulario". NO incluir email/teléfono en error_message.</t>
         </is>
       </c>
+      <c r="M8" s="4" t="inlineStr">
+        <is>
+          <t>track('form_error', { form_id: 'calculator', error_code: String(err.status), error_message: err.code });</t>
+        </is>
+      </c>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>Catch del fetch/axios del submit. Mandar SOLO códigos, NO el body completo (puede llevar PII).</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1258,6 +1342,16 @@
           <t>Sustituye al "Campo actualizado: {field}" (que era ruido). Solo se dispara en error de validación.</t>
         </is>
       </c>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t>track('form_field_error', { form_id: 'reservation', field_name: 'postal_code', error_type: 'invalid_format' });</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>Hook de validación (Yup/Zod/RHF): dentro del callback onError de cada campo, no en cada onChange.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1317,7 +1411,17 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>Sustituye al "Petición de Llamada Cancelada" y "Cancelar Registro".</t>
+          <t>Sustituye a "Petición de Llamada Cancelada" y "Cancelar Registro".</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t>track('form_cancel', { form_id: 'onlyphone', step: 'phone' });</t>
+        </is>
+      </c>
+      <c r="N10" s="4" t="inlineStr">
+        <is>
+          <t>onClick del botón cerrar/cancelar del modal, o en el unmount si form_start se disparó pero no hubo submit.</t>
         </is>
       </c>
     </row>
@@ -1382,6 +1486,16 @@
           <t>Marca como conversion en GA4. UNIFICA: "Formulario de Contacto Exitoso", "Envío Exitoso del Formulario", "Petición de Llamada Correcta" y "Reserva Completada". Duplicar server-side (ANL-9). NO email en label.</t>
         </is>
       </c>
+      <c r="M11" s="4" t="inlineStr">
+        <is>
+          <t>track('generate_lead', { form_id: 'reservation', lead_source: 'reservation', value: cartTotal, currency: 'EUR', items: cartItems });</t>
+        </is>
+      </c>
+      <c r="N11" s="4" t="inlineStr">
+        <is>
+          <t>Tras la respuesta 200 del POST al endpoint del formulario. NO en el onClick. Duplicar también en el backend (ver ANL-9 en ANALYTICS.md).</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1444,6 +1558,16 @@
           <t>Permite medir abandono entre llegada y primer add_to_cart.</t>
         </is>
       </c>
+      <c r="M12" s="4" t="inlineStr">
+        <is>
+          <t>track('view_calculator', { country });</t>
+        </is>
+      </c>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
+          <t>useEffect(() =&gt; { ... }, []) al montar el componente raíz de la calculadora.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1506,6 +1630,16 @@
           <t>Sustituye a "Artículo añadido al Resumen". CRÍTICO: la función del carrito existe pero NO se dispara hoy. Resolver en ANL-7.</t>
         </is>
       </c>
+      <c r="M13" s="4" t="inlineStr">
+        <is>
+          <t>track('add_to_cart', { currency: 'EUR', value: item.price * item.quantity, items: [toGA4Item(item)], context: 'cart' });</t>
+        </is>
+      </c>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
+          <t>Handler onAddItem de la calculadora Y onAddToCart del carrito principal (la utilidad ya existe en el repo, hay que llamarla).</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1568,6 +1702,16 @@
           <t>Sustituye a "Artículo eliminado del Resumen" y "Eliminar del Carrito".</t>
         </is>
       </c>
+      <c r="M14" s="4" t="inlineStr">
+        <is>
+          <t>track('remove_from_cart', { currency: 'EUR', value, items: [toGA4Item(removedItem)], context: 'cart' });</t>
+        </is>
+      </c>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t>Handler onRemove en los TRES sitios: resumen visible, dropdown del header y vista móvil.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1630,6 +1774,16 @@
           <t>Marca el inicio del checkout. Permite construir audiencia "carrito abandonado" en GA4 (begin_checkout sin generate_lead en 24h).</t>
         </is>
       </c>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>track('begin_checkout', { currency: 'EUR', value: cartTotal, items: cartItems });</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
+          <t>useEffect al montar la página de checkout/reserva, dentro de un if (cartItems.length &gt; 0).</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1692,6 +1846,16 @@
           <t>Sustituye a "Reserva Completada". Diferencia el click del envío confirmado (que es generate_lead).</t>
         </is>
       </c>
+      <c r="M16" s="4" t="inlineStr">
+        <is>
+          <t>track('begin_checkout_submit', { currency: 'EUR', value: cartTotal, items: cartItems });</t>
+        </is>
+      </c>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
+          <t>onClick del botón "Solicitar cotización", justo antes del fetch al backend (después de validar términos).</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1754,6 +1918,16 @@
           <t>Sustituye al "Formulario de Login Exitoso". NO email/nombre en label — pasar user_id hasheado.</t>
         </is>
       </c>
+      <c r="M17" s="4" t="inlineStr">
+        <is>
+          <t>track('login', { method: 'email', user_id: user.id });</t>
+        </is>
+      </c>
+      <c r="N17" s="4" t="inlineStr">
+        <is>
+          <t>Tras 200 OK del POST /api/login, una vez tienes el user.id de la respuesta.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1816,6 +1990,16 @@
           <t>Sustituye al "Formulario de Login Erróneo". NO email en label.</t>
         </is>
       </c>
+      <c r="M18" s="4" t="inlineStr">
+        <is>
+          <t>track('login_error', { method: 'email', error_code: err.code || String(err.status) });</t>
+        </is>
+      </c>
+      <c r="N18" s="4" t="inlineStr">
+        <is>
+          <t>Catch del POST /api/login. NO mandar email.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1878,6 +2062,16 @@
           <t>Sustituye a "Formulario de Registro Visto". Distinguir demandante (renter) de alquilador (partner).</t>
         </is>
       </c>
+      <c r="M19" s="4" t="inlineStr">
+        <is>
+          <t>track('sign_up_view', { user_type: 'renter', source: 'checkout' });</t>
+        </is>
+      </c>
+      <c r="N19" s="4" t="inlineStr">
+        <is>
+          <t>useEffect al montar el modal/página de registro. user_type viene del prop o del prop o de la ruta (/registro vs /alquiladores).</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1940,6 +2134,16 @@
           <t>Sustituye a "Formulario de Registro Exitoso". Marcar conversion solo cuando user_type=partner. Server-side en ANL-9.</t>
         </is>
       </c>
+      <c r="M20" s="4" t="inlineStr">
+        <is>
+          <t>track('sign_up', { method: 'email', user_type: 'partner', user_id: newUser.id });</t>
+        </is>
+      </c>
+      <c r="N20" s="4" t="inlineStr">
+        <is>
+          <t>Tras 200 OK del POST /api/signup. Llamar también a identify() para setear user_properties. Duplicar server-side (ANL-9).</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -2002,6 +2206,16 @@
           <t>Sustituye a "Formulario de Registro Erróneo".</t>
         </is>
       </c>
+      <c r="M21" s="4" t="inlineStr">
+        <is>
+          <t>track('sign_up_error', { method: 'email', user_type: 'renter', error_code: err.code });</t>
+        </is>
+      </c>
+      <c r="N21" s="4" t="inlineStr">
+        <is>
+          <t>Catch del POST /api/signup.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -2064,6 +2278,16 @@
           <t>Unifica "Cancelar Registro" y "Cerrar Registro Exitoso".</t>
         </is>
       </c>
+      <c r="M22" s="4" t="inlineStr">
+        <is>
+          <t>track('sign_up_cancel', { user_type: 'renter', step: 'form' });</t>
+        </is>
+      </c>
+      <c r="N22" s="4" t="inlineStr">
+        <is>
+          <t>onClick de cerrar el modal de registro (step='form') Y onClick de cerrar el mensaje de éxito (step='success_modal').</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -2126,6 +2350,16 @@
           <t>Unifica "Aceptar Términos" y "Desmarcar Términos" en uno con parámetro accepted.</t>
         </is>
       </c>
+      <c r="M23" s="4" t="inlineStr">
+        <is>
+          <t>track('terms_toggle', { accepted: e.target.checked, form_id: 'checkout' });</t>
+        </is>
+      </c>
+      <c r="N23" s="4" t="inlineStr">
+        <is>
+          <t>onChange del checkbox de términos en cualquier formulario.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -2188,6 +2422,16 @@
           <t>NUEVO. Hoy no se mide qué categorías/ubicaciones consulta el usuario.</t>
         </is>
       </c>
+      <c r="M24" s="4" t="inlineStr">
+        <is>
+          <t>track('view_item_list', { item_list_id: category.slug, item_list_name: category.name, items: products.map(toGA4Item) });</t>
+        </is>
+      </c>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
+          <t>useEffect al montar las páginas de listado (/alquiler/maquinaria/* y /ubicaciones/*) cuando ya están los items cargados.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -2250,6 +2494,16 @@
           <t>NUEVO. Permite funnel completo desde catálogo a lead.</t>
         </is>
       </c>
+      <c r="M25" s="4" t="inlineStr">
+        <is>
+          <t>track('view_item', { currency: 'EUR', items: [toGA4Item(product)] });</t>
+        </is>
+      </c>
+      <c r="N25" s="4" t="inlineStr">
+        <is>
+          <t>useEffect al montar la página de detalle de producto.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -2312,6 +2566,16 @@
           <t>NUEVO. Permite analizar posición/CTR de tarjetas.</t>
         </is>
       </c>
+      <c r="M26" s="4" t="inlineStr">
+        <is>
+          <t>track('select_item', { item_list_name: category.name, items: [{ ...toGA4Item(product), index: idx }] });</t>
+        </is>
+      </c>
+      <c r="N26" s="4" t="inlineStr">
+        <is>
+          <t>onClick de cada tarjeta de producto, antes de navegar.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -2374,6 +2638,16 @@
           <t>NUEVO. Útil para entender intención y mejorar UX.</t>
         </is>
       </c>
+      <c r="M27" s="4" t="inlineStr">
+        <is>
+          <t>track('filter_apply', { filter_type: 'location', filter_value: selectedValue, item_list_name });</t>
+        </is>
+      </c>
+      <c r="N27" s="4" t="inlineStr">
+        <is>
+          <t>onChange (con debounce 300ms) de cada control de filtro u ordenación.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -2436,6 +2710,16 @@
           <t>NUEVO. GA4 lo trae en Enhanced Measurement, pero conviene parametrizar destination_type para distinguir alquiladores.</t>
         </is>
       </c>
+      <c r="M28" s="4" t="inlineStr">
+        <is>
+          <t>track('click_outbound', { outbound_url: link.href, destination_type: 'rental_company' });</t>
+        </is>
+      </c>
+      <c r="N28" s="4" t="inlineStr">
+        <is>
+          <t>Mejor con event delegation global en _app.jsx/_layout: document.addEventListener('click', ...) filtrando por &lt;a target='_blank'&gt; o host distinto.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -2496,6 +2780,16 @@
       <c r="L29" s="4" t="inlineStr">
         <is>
           <t>NUEVO. Detecta enlaces rotos y errores de rutas.</t>
+        </is>
+      </c>
+      <c r="M29" s="4" t="inlineStr">
+        <is>
+          <t>track('page_not_found', { path: window.location.pathname, referrer: document.referrer });</t>
+        </is>
+      </c>
+      <c r="N29" s="4" t="inlineStr">
+        <is>
+          <t>useEffect en la plantilla 404 (pages/404.jsx o app/not-found.jsx en Next.js).</t>
         </is>
       </c>
     </row>

</xml_diff>